<commit_message>
PCB updated: Zero Errors
</commit_message>
<xml_diff>
--- a/Hardware/Components/Shield_BOM.xlsx
+++ b/Hardware/Components/Shield_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\aymen\My_Work\KiCadProjects\Shield_V1\Hardware\Components\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SyedAymen\Shield\Hardware\Components\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A2B6082-B4C4-46AD-A5A7-12E34EF1823B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6B4E66-D5D4-48B6-83E2-ECE303F8C3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="815" yWindow="-109" windowWidth="17851" windowHeight="10651" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="18775" windowHeight="10651" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="84">
   <si>
     <t>S. NO</t>
   </si>
@@ -279,6 +279,15 @@
   </si>
   <si>
     <t>MMBT3904-7-F</t>
+  </si>
+  <si>
+    <t>TXB0102DCUR - 2-Bit Bidirectional Voltage-Level Shifter Auto Direction Sensing 8-Pin VSSOP</t>
+  </si>
+  <si>
+    <t>UART-LTE-MCU</t>
+  </si>
+  <si>
+    <t>TXB0102DCUR</t>
   </si>
 </sst>
 </file>
@@ -1366,10 +1375,31 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="28.55" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="3">
+        <v>1</v>
+      </c>
+      <c r="F28" s="3">
+        <v>28</v>
+      </c>
       <c r="G28" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>28</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1400,8 +1430,9 @@
     <hyperlink ref="H25" r:id="rId24" xr:uid="{686EEFA9-2ACB-4929-BD4A-C3CD3700A705}"/>
     <hyperlink ref="H26" r:id="rId25" xr:uid="{680CBD2C-8F49-43D1-87D1-99FFF2CBAFCE}"/>
     <hyperlink ref="H27" r:id="rId26" xr:uid="{61788516-A217-4F10-A951-44E08A6CD277}"/>
+    <hyperlink ref="H28" r:id="rId27" xr:uid="{BDFD280E-B051-4D67-9FA8-D7568A76456D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId27"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId28"/>
 </worksheet>
 </file>
</xml_diff>